<commit_message>
Weekly full pipeline run — 2026-10-18
</commit_message>
<xml_diff>
--- a/data/master.xlsx
+++ b/data/master.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T375"/>
+  <dimension ref="A1:T381"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -26358,6 +26358,478 @@
       <c r="S375" t="inlineStr"/>
       <c r="T375" t="inlineStr"/>
     </row>
+    <row r="376">
+      <c r="A376" t="inlineStr">
+        <is>
+          <t>115195257449</t>
+        </is>
+      </c>
+      <c r="B376" t="inlineStr">
+        <is>
+          <t>2026-10-15T06:40:31+00:00</t>
+        </is>
+      </c>
+      <c r="C376" t="n">
+        <v>3</v>
+      </c>
+      <c r="D376" t="inlineStr">
+        <is>
+          <t>took a while to get the payment amount</t>
+        </is>
+      </c>
+      <c r="E376" t="inlineStr">
+        <is>
+          <t>Payments</t>
+        </is>
+      </c>
+      <c r="F376" t="inlineStr">
+        <is>
+          <t>Payments</t>
+        </is>
+      </c>
+      <c r="G376" t="inlineStr">
+        <is>
+          <t>Bugs/ glitch</t>
+        </is>
+      </c>
+      <c r="H376" t="inlineStr">
+        <is>
+          <t>Challenges and Workarounds</t>
+        </is>
+      </c>
+      <c r="I376" t="n">
+        <v>0.236</v>
+      </c>
+      <c r="J376" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="K376" t="inlineStr">
+        <is>
+          <t>[{"topic": "Payments", "detail": "payment, payment system, card payment", "sentiment": "negative", "confidence": 0.887, "source": "absa_aspect"}, {"topic": "Challenges and Workarounds", "detail": "crash, bug, error", "sentiment": "negative", "confidence": 0.954, "source": "absa_aspect"}]</t>
+        </is>
+      </c>
+      <c r="L376" t="inlineStr">
+        <is>
+          <t>payment, payment system, card payment, crash, bug, error</t>
+        </is>
+      </c>
+      <c r="M376" t="inlineStr">
+        <is>
+          <t>payment: negative (0.885), payment system: negative (0.887), card payment: negative (0.835), crash: negative (0.954), bug: negative (0.865), error: negative (0.896)</t>
+        </is>
+      </c>
+      <c r="N376" t="inlineStr">
+        <is>
+          <t>negative</t>
+        </is>
+      </c>
+      <c r="O376" t="inlineStr">
+        <is>
+          <t>negative</t>
+        </is>
+      </c>
+      <c r="P376" t="inlineStr"/>
+      <c r="Q376" t="inlineStr"/>
+      <c r="R376" t="inlineStr"/>
+      <c r="S376" t="inlineStr"/>
+      <c r="T376" t="inlineStr"/>
+    </row>
+    <row r="377">
+      <c r="A377" t="inlineStr">
+        <is>
+          <t>115195276206</t>
+        </is>
+      </c>
+      <c r="B377" t="inlineStr">
+        <is>
+          <t>2026-10-15T07:33:15+00:00</t>
+        </is>
+      </c>
+      <c r="C377" t="n">
+        <v>4</v>
+      </c>
+      <c r="D377" t="inlineStr">
+        <is>
+          <t>building control fees is confusing</t>
+        </is>
+      </c>
+      <c r="E377" t="inlineStr">
+        <is>
+          <t>Fees too high</t>
+        </is>
+      </c>
+      <c r="F377" t="inlineStr">
+        <is>
+          <t>Fees, charges and quotes</t>
+        </is>
+      </c>
+      <c r="G377" t="inlineStr">
+        <is>
+          <t>Confusing</t>
+        </is>
+      </c>
+      <c r="H377" t="inlineStr">
+        <is>
+          <t>Negative experience, Challenges and Workarounds</t>
+        </is>
+      </c>
+      <c r="I377" t="n">
+        <v>0.365</v>
+      </c>
+      <c r="J377" t="inlineStr">
+        <is>
+          <t>svm</t>
+        </is>
+      </c>
+      <c r="K377" t="inlineStr">
+        <is>
+          <t>[{"topic": "Fees, charges and quotes", "detail": "fees, charges, charge", "sentiment": "negative", "confidence": 0.889, "source": "absa_aspect"}, {"topic": "Challenges and Workarounds", "detail": "crash, bug, error", "sentiment": "negative", "confidence": 0.956, "source": "absa_aspect"}]</t>
+        </is>
+      </c>
+      <c r="L377" t="inlineStr">
+        <is>
+          <t>fees, charges, charge, crash, bug, error</t>
+        </is>
+      </c>
+      <c r="M377" t="inlineStr">
+        <is>
+          <t>fees: negative (0.889), charges: negative (0.7), charge: negative (0.692), crash: negative (0.956), bug: negative (0.873), error: negative (0.871)</t>
+        </is>
+      </c>
+      <c r="N377" t="inlineStr">
+        <is>
+          <t>negative</t>
+        </is>
+      </c>
+      <c r="O377" t="inlineStr">
+        <is>
+          <t>negative</t>
+        </is>
+      </c>
+      <c r="P377" t="inlineStr"/>
+      <c r="Q377" t="inlineStr"/>
+      <c r="R377" t="inlineStr"/>
+      <c r="S377" t="inlineStr"/>
+      <c r="T377" t="inlineStr"/>
+    </row>
+    <row r="378">
+      <c r="A378" t="inlineStr">
+        <is>
+          <t>115195472798</t>
+        </is>
+      </c>
+      <c r="B378" t="inlineStr">
+        <is>
+          <t>2026-10-15T14:07:06+00:00</t>
+        </is>
+      </c>
+      <c r="C378" t="n">
+        <v>2</v>
+      </c>
+      <c r="D378" t="inlineStr">
+        <is>
+          <t>when i nominate the client to pay the fee it asks for their email and my namecompany and i keep getting an email to say that i have been nominated to pay it does not put me in as a cc so i never know whether an email has been sent to the client</t>
+        </is>
+      </c>
+      <c r="E378" t="inlineStr">
+        <is>
+          <t>Nominations</t>
+        </is>
+      </c>
+      <c r="F378" t="inlineStr">
+        <is>
+          <t>Payments</t>
+        </is>
+      </c>
+      <c r="G378" t="inlineStr">
+        <is>
+          <t>Payments</t>
+        </is>
+      </c>
+      <c r="H378" t="inlineStr">
+        <is>
+          <t>Payments, Missing features &amp; feature requests, Challenges and Workarounds</t>
+        </is>
+      </c>
+      <c r="I378" t="n">
+        <v>0.251</v>
+      </c>
+      <c r="J378" t="inlineStr">
+        <is>
+          <t>override</t>
+        </is>
+      </c>
+      <c r="K378" t="inlineStr">
+        <is>
+          <t>[{"topic": "Payments", "detail": "payment, card payment", "sentiment": "neutral", "confidence": 0.991, "source": "absa_aspect"}, {"topic": "Missing features &amp; feature requests", "detail": "missing feature, suggestion, improvement", "sentiment": "negative", "confidence": 0.748, "source": "absa_aspect"}, {"topic": "Challenges and Workarounds", "detail": "error", "sentiment": "negative", "confidence": 0.641, "source": "absa_aspect"}]</t>
+        </is>
+      </c>
+      <c r="L378" t="inlineStr">
+        <is>
+          <t>payment, card payment, missing feature, suggestion, improvement, error</t>
+        </is>
+      </c>
+      <c r="M378" t="inlineStr">
+        <is>
+          <t>payment: neutral (0.991), card payment: neutral (0.949), missing feature: negative (0.732), suggestion: neutral (0.692), improvement: negative (0.748), error: negative (0.641)</t>
+        </is>
+      </c>
+      <c r="N378" t="inlineStr">
+        <is>
+          <t>negative</t>
+        </is>
+      </c>
+      <c r="O378" t="inlineStr">
+        <is>
+          <t>negative</t>
+        </is>
+      </c>
+      <c r="P378" t="inlineStr"/>
+      <c r="Q378" t="inlineStr"/>
+      <c r="R378" t="inlineStr"/>
+      <c r="S378" t="inlineStr"/>
+      <c r="T378" t="inlineStr"/>
+    </row>
+    <row r="379">
+      <c r="A379" t="inlineStr">
+        <is>
+          <t>115196004105</t>
+        </is>
+      </c>
+      <c r="B379" t="inlineStr">
+        <is>
+          <t>2026-10-16T06:18:21+00:00</t>
+        </is>
+      </c>
+      <c r="C379" t="n">
+        <v>3</v>
+      </c>
+      <c r="D379" t="inlineStr">
+        <is>
+          <t>some of the questions are written in a way that someone who doesnt regularly deal with planning issues cant understand</t>
+        </is>
+      </c>
+      <c r="E379" t="inlineStr">
+        <is>
+          <t>Confusing</t>
+        </is>
+      </c>
+      <c r="F379" t="inlineStr">
+        <is>
+          <t>Negative experience</t>
+        </is>
+      </c>
+      <c r="G379" t="inlineStr"/>
+      <c r="H379" t="inlineStr">
+        <is>
+          <t>Guidance, clarity &amp; jargon, Challenges and Workarounds, Missing features &amp; feature requests</t>
+        </is>
+      </c>
+      <c r="I379" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="J379" t="inlineStr">
+        <is>
+          <t>svm_low_conf</t>
+        </is>
+      </c>
+      <c r="K379" t="inlineStr">
+        <is>
+          <t>[{"topic": "Guidance, clarity &amp; jargon", "detail": "guidance, instructions, jargon", "sentiment": "negative", "confidence": 0.985, "source": "absa_aspect"}, {"topic": "Challenges and Workarounds", "detail": "crash, bug, error", "sentiment": "negative", "confidence": 0.889, "source": "absa_aspect"}, {"topic": "Missing features &amp; feature requests", "detail": "missing feature, suggestion, improvement", "sentiment": "negative", "confidence": 0.854, "source": "absa_aspect"}]</t>
+        </is>
+      </c>
+      <c r="L379" t="inlineStr">
+        <is>
+          <t>guidance, instructions, jargon, crash, bug, error, missing feature, suggestion, improvement</t>
+        </is>
+      </c>
+      <c r="M379" t="inlineStr">
+        <is>
+          <t>guidance: neutral (0.951), instructions: neutral (0.934), jargon: negative (0.985), crash: neutral (0.803), bug: negative (0.889), error: negative (0.874), missing feature: negative (0.854), suggestion: neutral (0.774), improvement: negative (0.722)</t>
+        </is>
+      </c>
+      <c r="N379" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="O379" t="inlineStr">
+        <is>
+          <t>negative</t>
+        </is>
+      </c>
+      <c r="P379" t="inlineStr"/>
+      <c r="Q379" t="inlineStr"/>
+      <c r="R379" t="inlineStr"/>
+      <c r="S379" t="inlineStr"/>
+      <c r="T379" t="inlineStr">
+        <is>
+          <t>frequent</t>
+        </is>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" t="inlineStr">
+        <is>
+          <t>115196141267</t>
+        </is>
+      </c>
+      <c r="B380" t="inlineStr">
+        <is>
+          <t>2026-10-16T12:08:13+00:00</t>
+        </is>
+      </c>
+      <c r="C380" t="n">
+        <v>1</v>
+      </c>
+      <c r="D380" t="inlineStr">
+        <is>
+          <t>bristol council allow one full payment instead of two staged payments  but this option was not available so you get an extra £40 for me to not bother arguing with you well done</t>
+        </is>
+      </c>
+      <c r="E380" t="inlineStr">
+        <is>
+          <t>Payments</t>
+        </is>
+      </c>
+      <c r="F380" t="inlineStr">
+        <is>
+          <t>Payments</t>
+        </is>
+      </c>
+      <c r="G380" t="inlineStr"/>
+      <c r="H380" t="inlineStr">
+        <is>
+          <t>Fees, charges and quotes</t>
+        </is>
+      </c>
+      <c r="I380" t="n">
+        <v>0.152</v>
+      </c>
+      <c r="J380" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="K380" t="inlineStr">
+        <is>
+          <t>[{"topic": "Payments", "detail": "payment, payment system, card payment", "sentiment": "neutral", "confidence": 0.873, "source": "absa_aspect"}, {"topic": "Fees, charges and quotes", "detail": "charges", "sentiment": "negative", "confidence": 0.606, "source": "absa_aspect"}]</t>
+        </is>
+      </c>
+      <c r="L380" t="inlineStr">
+        <is>
+          <t>payment, payment system, card payment, charges</t>
+        </is>
+      </c>
+      <c r="M380" t="inlineStr">
+        <is>
+          <t>payment: neutral (0.873), payment system: negative (0.841), card payment: neutral (0.839), charges: negative (0.606)</t>
+        </is>
+      </c>
+      <c r="N380" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="O380" t="inlineStr">
+        <is>
+          <t>negative</t>
+        </is>
+      </c>
+      <c r="P380" t="inlineStr">
+        <is>
+          <t>Bristol</t>
+        </is>
+      </c>
+      <c r="Q380" t="inlineStr"/>
+      <c r="R380" t="inlineStr"/>
+      <c r="S380" t="inlineStr">
+        <is>
+          <t>£40</t>
+        </is>
+      </c>
+      <c r="T380" t="inlineStr"/>
+    </row>
+    <row r="381">
+      <c r="A381" t="inlineStr">
+        <is>
+          <t>115196217061</t>
+        </is>
+      </c>
+      <c r="B381" t="inlineStr">
+        <is>
+          <t>2026-10-16T14:13:49+00:00</t>
+        </is>
+      </c>
+      <c r="C381" t="n">
+        <v>1</v>
+      </c>
+      <c r="D381" t="inlineStr">
+        <is>
+          <t>difficulty at your end  had to reset the application</t>
+        </is>
+      </c>
+      <c r="E381" t="inlineStr">
+        <is>
+          <t>Negative experience</t>
+        </is>
+      </c>
+      <c r="F381" t="inlineStr">
+        <is>
+          <t>Negative experience</t>
+        </is>
+      </c>
+      <c r="G381" t="inlineStr">
+        <is>
+          <t>Bugs/ glitch</t>
+        </is>
+      </c>
+      <c r="H381" t="inlineStr">
+        <is>
+          <t>Challenges and Workarounds</t>
+        </is>
+      </c>
+      <c r="I381" t="n">
+        <v>0.268</v>
+      </c>
+      <c r="J381" t="inlineStr">
+        <is>
+          <t>svm_low_conf</t>
+        </is>
+      </c>
+      <c r="K381" t="inlineStr">
+        <is>
+          <t>[{"topic": "Challenges and Workarounds", "detail": "crash, bug, error", "sentiment": "negative", "confidence": 0.995, "source": "absa_aspect"}]</t>
+        </is>
+      </c>
+      <c r="L381" t="inlineStr">
+        <is>
+          <t>crash, bug, error</t>
+        </is>
+      </c>
+      <c r="M381" t="inlineStr">
+        <is>
+          <t>crash: negative (0.995), bug: negative (0.984), error: negative (0.984)</t>
+        </is>
+      </c>
+      <c r="N381" t="inlineStr">
+        <is>
+          <t>negative</t>
+        </is>
+      </c>
+      <c r="O381" t="inlineStr">
+        <is>
+          <t>negative</t>
+        </is>
+      </c>
+      <c r="P381" t="inlineStr"/>
+      <c r="Q381" t="inlineStr"/>
+      <c r="R381" t="inlineStr"/>
+      <c r="S381" t="inlineStr"/>
+      <c r="T381" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>